<commit_message>
"Update `metrics_dashboard.json` to reflect latest financial data and timestamp, ensuring alignment with current sector-wise and aggregated metrics."
Signed-off-by: Kabenge42 <mmutaaga@gmail.com>
</commit_message>
<xml_diff>
--- a/outputs/eda/phase93_category_analysis_report.xlsx
+++ b/outputs/eda/phase93_category_analysis_report.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6971</v>
+        <v>6976</v>
       </c>
     </row>
     <row r="3">
@@ -703,37 +703,37 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.03323940633069485</v>
+        <v>-0.05159207565659022</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.07605384612552675</v>
+        <v>-0.06240387652834602</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0236102407506419</v>
+        <v>-0.02787014997543389</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.03697729618650481</v>
+        <v>-0.05648429343327727</v>
       </c>
       <c r="F2" t="n">
-        <v>0.004243397697943961</v>
+        <v>-0.01004255843608416</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05349654688905923</v>
+        <v>0.04720220520972962</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0280884891327617</v>
+        <v>0.05913734693114382</v>
       </c>
       <c r="I2" t="n">
-        <v>-0.03228926387750927</v>
+        <v>-0.01022878197325005</v>
       </c>
       <c r="J2" t="n">
-        <v>0.07603816045230452</v>
+        <v>0.07150945984075827</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.08475603281343701</v>
+        <v>-0.06145744981315441</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.04708808678554304</v>
+        <v>-0.08493765700429136</v>
       </c>
     </row>
     <row r="3">
@@ -743,37 +743,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.01199009660155664</v>
+        <v>-0.0114769031628928</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.07324473048640462</v>
+        <v>-0.07761397775769154</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.07573964898120798</v>
+        <v>-0.08236469037910324</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.08688093956933064</v>
+        <v>-0.1184198261740697</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1298532863468034</v>
+        <v>-0.128506269132784</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2464441529388045</v>
+        <v>0.2319140188646223</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.03788830416021713</v>
+        <v>-0.03043506700311878</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2119915434005649</v>
+        <v>0.2411065532214795</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.01702164430727116</v>
+        <v>-0.0122435139027342</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.01043987782774995</v>
+        <v>0.03378455360708189</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.09764976425732927</v>
+        <v>-0.09139772703357034</v>
       </c>
     </row>
     <row r="4">
@@ -783,37 +783,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.209938709580605</v>
+        <v>0.2041819286780852</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.04734194206232502</v>
+        <v>-0.04906771981025451</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.05275828380408373</v>
+        <v>-0.0422735804277948</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2000416988106282</v>
+        <v>0.17742771550524</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1353048453701994</v>
+        <v>0.1304086936089322</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01778965666853598</v>
+        <v>0.01952538416408754</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.1108785996544071</v>
+        <v>-0.1131466726869313</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01529449177164545</v>
+        <v>-0.002553771510810373</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.1168857546389333</v>
+        <v>-0.1157876247211264</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.04294158777873049</v>
+        <v>-0.03707573163117359</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0473718834770298</v>
+        <v>0.03510876728747487</v>
       </c>
     </row>
     <row r="5">
@@ -823,37 +823,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.02519736325745504</v>
+        <v>-0.02623295096592201</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0004590587566864648</v>
+        <v>-0.005449278829940542</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1359638271729208</v>
+        <v>-0.132724378708595</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01143316021530266</v>
+        <v>-0.004066010144512008</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.01520321347765285</v>
+        <v>-0.01722267754902901</v>
       </c>
       <c r="G5" t="n">
-        <v>0.01877552119218129</v>
+        <v>0.01133067885796123</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.01747788693914597</v>
+        <v>-0.01771437765853444</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1500024747128878</v>
+        <v>0.1866602472584065</v>
       </c>
       <c r="J5" t="n">
-        <v>0.02626644986962418</v>
+        <v>0.03063443157824903</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.1914779460624793</v>
+        <v>-0.1959366367410036</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.008566565891308596</v>
+        <v>-0.07606786175283266</v>
       </c>
     </row>
     <row r="6">
@@ -863,37 +863,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02385896308975414</v>
+        <v>0.02649429582314388</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00768690324971629</v>
+        <v>0.01012783838077674</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0162830904294665</v>
+        <v>0.02119977310068383</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01073752330279884</v>
+        <v>0.01237260993888548</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.05884913169645231</v>
+        <v>-0.06235003520873695</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02060680728108662</v>
+        <v>0.02347062954123512</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01107119666484912</v>
+        <v>0.01262258736880096</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01956046890003891</v>
+        <v>0.01958567352150811</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0002457299896175378</v>
+        <v>0.003062651723569088</v>
       </c>
       <c r="K6" t="n">
-        <v>0.009480041128061327</v>
+        <v>0.0100456904648159</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.05300915998102019</v>
+        <v>-0.05014889561816557</v>
       </c>
     </row>
     <row r="7">
@@ -903,37 +903,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.009846218995920719</v>
+        <v>-0.02126988284390626</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.008887323494928758</v>
+        <v>0.01183236319883222</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.02794148177098256</v>
+        <v>-0.01986991109656255</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1595405597253971</v>
+        <v>0.139597758648848</v>
       </c>
       <c r="F7" t="n">
-        <v>0.03832889250997865</v>
+        <v>0.007530003875411424</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03534515490938154</v>
+        <v>0.01567928194343775</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.02389876869899855</v>
+        <v>-0.01601875530780573</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0005382353863348838</v>
+        <v>0.02026343653764697</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.03384521678495105</v>
+        <v>-0.02483813561487978</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.1163157912973105</v>
+        <v>-0.1204450926407142</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.02904320159939766</v>
+        <v>-0.0345136864985234</v>
       </c>
     </row>
   </sheetData>
@@ -994,22 +994,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.03355094509149489</v>
+        <v>-0.06391598946391759</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.1345855359883626</v>
+        <v>-0.1371838244077556</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.09394404687206459</v>
+        <v>-0.1178724652238784</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1173992778512986</v>
+        <v>-0.1171542348750286</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.006371388649674462</v>
+        <v>-0.003658035540172609</v>
       </c>
       <c r="G2" t="n">
-        <v>0.02255839035932099</v>
+        <v>-0.01090781355230613</v>
       </c>
     </row>
     <row r="3">
@@ -1019,22 +1019,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1018457300355783</v>
+        <v>0.1324996163481542</v>
       </c>
       <c r="C3" t="n">
-        <v>0.03809381047951223</v>
+        <v>0.06044095710271572</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.07259421133796472</v>
+        <v>-0.02500511892872506</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.01061249181822044</v>
+        <v>0.01486589782324356</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.01580313626985895</v>
+        <v>-0.02077411911885218</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.03613315968705465</v>
+        <v>0.03427991273044029</v>
       </c>
     </row>
     <row r="4">
@@ -1044,22 +1044,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.07656429150965524</v>
+        <v>-0.08224180534579188</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.03756505366790357</v>
+        <v>-0.05517248575537825</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.003304512907662505</v>
+        <v>-0.01924765706102244</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.04221872638018805</v>
+        <v>-0.05029760437386869</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0002113896628203643</v>
+        <v>0.003852061753294852</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.06656125923564274</v>
+        <v>-0.08724269401724445</v>
       </c>
     </row>
     <row r="5">
@@ -1069,22 +1069,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.01471399725303171</v>
+        <v>-0.02025496213398987</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.1465240559889474</v>
+        <v>-0.1495285226535372</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.07255749643492582</v>
+        <v>-0.09100101796472822</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.03307082577633177</v>
+        <v>-0.03913699645274384</v>
       </c>
       <c r="F5" t="n">
-        <v>0.007281279005503789</v>
+        <v>0.008636983528893629</v>
       </c>
       <c r="G5" t="n">
-        <v>0.003289005946433548</v>
+        <v>-0.03178761887985342</v>
       </c>
     </row>
     <row r="6">
@@ -1094,22 +1094,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.01792143103709907</v>
+        <v>-0.02809834347259031</v>
       </c>
       <c r="C6" t="n">
-        <v>0.08087958942976534</v>
+        <v>0.07725465233137141</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1373250817675861</v>
+        <v>0.1145743794898532</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1129631821057575</v>
+        <v>0.09409327617853611</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01883772610250119</v>
+        <v>0.01901039666147995</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1076033812311243</v>
+        <v>0.07073395160637271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>